<commit_message>
Fixed component testbench ports, initial printf C test programs, file handling update for raw pipeline dumping
</commit_message>
<xml_diff>
--- a/docs/spreadsheets/csr_spec.xlsx
+++ b/docs/spreadsheets/csr_spec.xlsx
@@ -100,22 +100,22 @@
     <t xml:space="preserve">machine status register (currently only used for testing)</t>
   </si>
   <si>
+    <t xml:space="preserve">mdbg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7A0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom register for holding debug info during testing</t>
+  </si>
+  <si>
     <t xml:space="preserve">mtest_status</t>
   </si>
   <si>
     <t xml:space="preserve">7C0</t>
   </si>
   <si>
-    <t xml:space="preserve">Custom Register for handelling test success/failure in simulation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mdbg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Custom register for holding debug info during testing</t>
+    <t xml:space="preserve">Custom register for handling test success/failure in simulation</t>
   </si>
 </sst>
 </file>
@@ -148,12 +148,18 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00A933"/>
+        <bgColor rgb="FF008000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -190,8 +196,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -208,6 +218,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF00A933"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -217,33 +287,37 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="53.11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -335,7 +409,7 @@
       <c r="F5" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>